<commit_message>
Update master route system and project list
</commit_message>
<xml_diff>
--- a/other/Projects.xlsx
+++ b/other/Projects.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\projects\Oahu\repo_new_model\other\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B756EF66-384F-4087-8FDD-5BE2C6242A4D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E6B6B7E1-593C-4605-B848-FA400C0F5DC3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-16356" yWindow="9000" windowWidth="16080" windowHeight="9660" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-16440" yWindow="1308" windowWidth="16080" windowHeight="9660" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Roadway" sheetId="1" r:id="rId1"/>
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="83" uniqueCount="57">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="89" uniqueCount="61">
   <si>
     <t>Waianae, Second Access, Farrington Highway to Kunia Road</t>
   </si>
@@ -198,6 +198,18 @@
   </si>
   <si>
     <t>OC-31-X16</t>
+  </si>
+  <si>
+    <t>Ewa/Mililani Busway Improvements - Fort Weaver Rd (Queens Medical Center West Oahu &amp; North Rd)</t>
+  </si>
+  <si>
+    <t>OC-31-108</t>
+  </si>
+  <si>
+    <t>Nimitz Busway Improvements - H-1 &amp; Bishop St</t>
+  </si>
+  <si>
+    <t>OC-31-96</t>
   </si>
 </sst>
 </file>
@@ -767,10 +779,11 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E065042F-84D0-4587-93CB-E2E810346385}">
-  <dimension ref="A1:E10"/>
+  <dimension ref="A1:E12"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="2" max="2" width="58.44140625" customWidth="1"/>
+    <col min="3" max="3" width="11.21875" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.3">
@@ -914,6 +927,34 @@
       </c>
       <c r="D10" t="s">
         <v>28</v>
+      </c>
+    </row>
+    <row r="11" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A11">
+        <v>9021</v>
+      </c>
+      <c r="B11" t="s">
+        <v>57</v>
+      </c>
+      <c r="C11" t="s">
+        <v>58</v>
+      </c>
+      <c r="D11" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="12" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A12">
+        <v>9022</v>
+      </c>
+      <c r="B12" t="s">
+        <v>59</v>
+      </c>
+      <c r="C12" t="s">
+        <v>60</v>
+      </c>
+      <c r="D12" t="s">
+        <v>21</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Add Kapolei to UH rail line
</commit_message>
<xml_diff>
--- a/other/Projects.xlsx
+++ b/other/Projects.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29328"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29530"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\projects\Oahu\repo_new_model\other\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E6B6B7E1-593C-4605-B848-FA400C0F5DC3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F6B4E06B-9C89-483D-A093-762E3F9F1AA3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-16440" yWindow="1308" windowWidth="16080" windowHeight="9660" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-15540" yWindow="10632" windowWidth="12960" windowHeight="9240" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Roadway" sheetId="1" r:id="rId1"/>
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="89" uniqueCount="61">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="90" uniqueCount="62">
   <si>
     <t>Waianae, Second Access, Farrington Highway to Kunia Road</t>
   </si>
@@ -210,6 +210,9 @@
   </si>
   <si>
     <t>OC-31-96</t>
+  </si>
+  <si>
+    <t>Fixed Guideway, Kapolei to UH</t>
   </si>
 </sst>
 </file>
@@ -779,7 +782,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E065042F-84D0-4587-93CB-E2E810346385}">
-  <dimension ref="A1:E12"/>
+  <dimension ref="A1:E13"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="2" max="2" width="58.44140625" customWidth="1"/>
@@ -955,6 +958,14 @@
       </c>
       <c r="D12" t="s">
         <v>21</v>
+      </c>
+    </row>
+    <row r="13" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A13">
+        <v>9023</v>
+      </c>
+      <c r="B13" t="s">
+        <v>61</v>
       </c>
     </row>
   </sheetData>

</xml_diff>